<commit_message>
Changed to LM5106 gate driver. Updated code for assymetric drive. Update LS math to account for dead time losses to through body diode instead of assuming transition losses as they don't exist in this architecture. Generated new list of mosfets
</commit_message>
<xml_diff>
--- a/Mosfet_extraction_pipeline/excel_sheets/High_side_frequency_optimization_matrix__LM5106.xlsx
+++ b/Mosfet_extraction_pipeline/excel_sheets/High_side_frequency_optimization_matrix__LM5106.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sync_Buck_convertor\Mosfet_extraction_pipeline\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sync_Buck_convertor\Mosfet_extraction_pipeline\excel_sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A503EE73-8468-4FCF-9C53-4B0876B9B743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2402F663-9E2D-490E-B476-AACB81C6E8F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,13 @@
     <t>Qg_nC</t>
   </si>
   <si>
+    <t>Ratio</t>
+  </si>
+  <si>
     <t>Infineon IAUCN04S7N054H</t>
+  </si>
+  <si>
+    <t>Infineon IAUCN04S7N040H</t>
   </si>
   <si>
     <t>Infineon IQE020N04LM6CG</t>
@@ -55,16 +61,13 @@
     <t>Infineon IQE020N04LM6CGSC</t>
   </si>
   <si>
+    <t>Infineon ISC058N04NM5</t>
+  </si>
+  <si>
     <t>onsemi NVMYS9D3N06CL</t>
   </si>
   <si>
-    <t>Infineon IAUCN04S7N040H</t>
-  </si>
-  <si>
     <t>Diodes Incorporated DMTH47M2SK3</t>
-  </si>
-  <si>
-    <t>Infineon ISC058N04NM5</t>
   </si>
   <si>
     <t>Infineon IAUCN04S7N047G</t>
@@ -84,26 +87,18 @@
   <si>
     <t>Infineon BSO220N03MD G</t>
   </si>
-  <si>
-    <t>Qg/Qsw</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -120,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -128,30 +123,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -458,39 +435,36 @@
   <dimension ref="A1:I146"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="16.08984375" customWidth="1"/>
-    <col min="5" max="5" width="17.90625" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" customWidth="1"/>
+    <col min="3" max="3" width="36.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>21</v>
+      <c r="I1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -501,10 +475,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>7.2068898809523829E-2</v>
+        <v>6.6705287247474751E-2</v>
       </c>
       <c r="E2">
         <v>9.0000000000000011E-3</v>
@@ -530,25 +504,25 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3">
-        <v>8.0168898809523811E-2</v>
+        <v>7.4149416035353535E-2</v>
       </c>
       <c r="E3">
-        <v>2.5000000000000001E-2</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="F3">
-        <v>2.0499999999999998</v>
+        <v>4.01</v>
       </c>
       <c r="G3">
-        <v>4.9000000000000004</v>
+        <v>5</v>
       </c>
       <c r="H3">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I3">
-        <v>5.1020408163265296</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -559,10 +533,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4">
-        <v>8.0168898809523811E-2</v>
+        <v>7.4165640782828279E-2</v>
       </c>
       <c r="E4">
         <v>2.5000000000000001E-2</v>
@@ -588,25 +562,25 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5">
-        <v>8.0426619047619052E-2</v>
+        <v>7.4165640782828279E-2</v>
       </c>
       <c r="E5">
-        <v>9.4999999999999998E-3</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="F5">
-        <v>9.1999999999999993</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="G5">
-        <v>1.8</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="H5">
-        <v>9.5</v>
+        <v>25</v>
       </c>
       <c r="I5">
-        <v>5.28</v>
+        <v>5.1020408163265296</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -617,25 +591,25 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>7.575726010101011E-2</v>
+      </c>
+      <c r="E6">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F6">
+        <v>5.8</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
         <v>12</v>
       </c>
-      <c r="D6">
-        <v>8.0798065476190478E-2</v>
-      </c>
-      <c r="E6">
-        <v>1.2999999999999999E-2</v>
-      </c>
-      <c r="F6">
-        <v>4.01</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>13</v>
-      </c>
       <c r="I6">
-        <v>2.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -646,10 +620,10 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7">
-        <v>8.1975148809523821E-2</v>
+        <v>7.5639315025252535E-2</v>
       </c>
       <c r="E7">
         <v>1.125E-2</v>
@@ -675,10 +649,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D8">
-        <v>8.6740119047619052E-2</v>
+        <v>8.1732272727272723E-2</v>
       </c>
       <c r="E8">
         <v>1.1875E-2</v>
@@ -704,10 +678,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>9.1812678571428566E-2</v>
+        <v>8.574046085858586E-2</v>
       </c>
       <c r="E9">
         <v>1.5125E-2</v>
@@ -733,10 +707,10 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10">
-        <v>9.3532738095238099E-2</v>
+        <v>8.6396148989898988E-2</v>
       </c>
       <c r="E10">
         <v>1.4999999999999999E-2</v>
@@ -762,10 +736,10 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11">
-        <v>9.498556547619047E-2</v>
+        <v>8.6948027146464643E-2</v>
       </c>
       <c r="E11">
         <v>1.6250000000000001E-2</v>
@@ -791,10 +765,10 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12">
-        <v>9.1881398809523812E-2</v>
+        <v>8.4573342803030319E-2</v>
       </c>
       <c r="E12">
         <v>1.35E-2</v>
@@ -820,10 +794,10 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D13">
-        <v>9.3053619047619052E-2</v>
+        <v>8.7545772727272736E-2</v>
       </c>
       <c r="E13">
         <v>1.4250000000000001E-2</v>
@@ -849,10 +823,10 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D14">
-        <v>0.10117967857142859</v>
+        <v>9.4301905303030314E-2</v>
       </c>
       <c r="E14">
         <v>1.8149999999999999E-2</v>
@@ -878,10 +852,10 @@
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D15">
-        <v>0.1052827380952381</v>
+        <v>9.7035037878787866E-2</v>
       </c>
       <c r="E15">
         <v>1.7999999999999999E-2</v>
@@ -907,10 +881,10 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D16">
-        <v>0.1091730654761905</v>
+        <v>9.9746638257575751E-2</v>
       </c>
       <c r="E16">
         <v>1.95E-2</v>
@@ -936,10 +910,10 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D17">
-        <v>9.9367119047619051E-2</v>
+        <v>9.3359272727272735E-2</v>
       </c>
       <c r="E17">
         <v>1.6625000000000001E-2</v>
@@ -965,10 +939,10 @@
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D18">
-        <v>0.1017876488095238</v>
+        <v>9.3507370580808089E-2</v>
       </c>
       <c r="E18">
         <v>1.575E-2</v>
@@ -994,10 +968,10 @@
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D19">
-        <v>0.11054667857142859</v>
+        <v>0.1028633497474747</v>
       </c>
       <c r="E19">
         <v>2.1174999999999999E-2</v>
@@ -1023,10 +997,10 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D20">
-        <v>0.11703273809523811</v>
+        <v>0.1076739267676768</v>
       </c>
       <c r="E20">
         <v>2.1000000000000001E-2</v>
@@ -1052,10 +1026,10 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21">
-        <v>0.12290476190476191</v>
+        <v>0.1124846906565657</v>
       </c>
       <c r="E21">
         <v>2.2749999999999999E-2</v>
@@ -1081,10 +1055,10 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D22">
-        <v>0.10568061904761911</v>
+        <v>9.9172772727272734E-2</v>
       </c>
       <c r="E22">
         <v>1.9E-2</v>
@@ -1110,10 +1084,10 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23">
-        <v>0.1116938988095238</v>
+        <v>0.1024413983585859</v>
       </c>
       <c r="E23">
         <v>1.7999999999999999E-2</v>
@@ -1139,10 +1113,10 @@
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D24">
-        <v>0.11991367857142859</v>
+        <v>0.1114247941919192</v>
       </c>
       <c r="E24">
         <v>2.4199999999999999E-2</v>
@@ -1168,10 +1142,10 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D25">
-        <v>0.1287827380952381</v>
+        <v>0.11831281565656571</v>
       </c>
       <c r="E25">
         <v>2.4E-2</v>
@@ -1200,22 +1174,22 @@
         <v>16</v>
       </c>
       <c r="D26">
-        <v>0.13600014285714279</v>
+        <v>0.1247103851010101</v>
       </c>
       <c r="E26">
-        <v>2.480000000000001E-2</v>
+        <v>2.5999999999999999E-2</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>4.7</v>
       </c>
       <c r="G26">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="H26">
-        <v>12.4</v>
+        <v>13</v>
       </c>
       <c r="I26">
-        <v>2.88</v>
+        <v>2.76595744680851</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -1226,10 +1200,10 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D27">
-        <v>0.11199411904761911</v>
+        <v>0.10498627272727271</v>
       </c>
       <c r="E27">
         <v>2.1375000000000002E-2</v>
@@ -1255,10 +1229,10 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D28">
-        <v>0.1216001488095238</v>
+        <v>0.1113754261363637</v>
       </c>
       <c r="E28">
         <v>2.0250000000000001E-2</v>
@@ -1284,10 +1258,10 @@
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D29">
-        <v>0.12928067857142861</v>
+        <v>0.1199862386363636</v>
       </c>
       <c r="E29">
         <v>2.7224999999999999E-2</v>
@@ -1313,10 +1287,10 @@
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D30">
-        <v>0.14053273809523811</v>
+        <v>0.12895170454545449</v>
       </c>
       <c r="E30">
         <v>2.7E-2</v>
@@ -1342,10 +1316,10 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D31">
-        <v>0.14850239285714281</v>
+        <v>0.1361168409090909</v>
       </c>
       <c r="E31">
         <v>2.7900000000000001E-2</v>
@@ -1371,10 +1345,10 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D32">
-        <v>0.11830761904761911</v>
+        <v>0.11079977272727271</v>
       </c>
       <c r="E32">
         <v>2.375E-2</v>
@@ -1400,10 +1374,10 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D33">
-        <v>0.13150639880952381</v>
+        <v>0.1203094539141414</v>
       </c>
       <c r="E33">
         <v>2.2499999999999999E-2</v>
@@ -1429,10 +1403,10 @@
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D34">
-        <v>0.1386476785714286</v>
+        <v>0.12854768308080811</v>
       </c>
       <c r="E34">
         <v>3.0249999999999999E-2</v>
@@ -1458,10 +1432,10 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D35">
-        <v>0.1522827380952381</v>
+        <v>0.13959059343434341</v>
       </c>
       <c r="E35">
         <v>0.03</v>
@@ -1487,10 +1461,10 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D36">
-        <v>0.16100464285714289</v>
+        <v>0.14742464646464651</v>
       </c>
       <c r="E36">
         <v>3.100000000000001E-2</v>
@@ -1516,10 +1490,10 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D37">
-        <v>0.12462111904761911</v>
+        <v>0.1166132727272727</v>
       </c>
       <c r="E37">
         <v>2.6124999999999999E-2</v>
@@ -1545,10 +1519,10 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D38">
-        <v>0.14141264880952381</v>
+        <v>0.12924348169191921</v>
       </c>
       <c r="E38">
         <v>2.4750000000000001E-2</v>
@@ -1574,10 +1548,10 @@
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D39">
-        <v>0.14801467857142861</v>
+        <v>0.13710912752525251</v>
       </c>
       <c r="E39">
         <v>3.3275000000000013E-2</v>
@@ -1603,10 +1577,10 @@
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40">
-        <v>0.16403273809523811</v>
+        <v>0.1502294823232323</v>
       </c>
       <c r="E40">
         <v>3.3000000000000002E-2</v>
@@ -1632,10 +1606,10 @@
         <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D41">
-        <v>0.17350689285714291</v>
+        <v>0.158732452020202</v>
       </c>
       <c r="E41">
         <v>3.4100000000000012E-2</v>
@@ -1661,10 +1635,10 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D42">
-        <v>0.13093461904761911</v>
+        <v>0.1224267727272727</v>
       </c>
       <c r="E42">
         <v>2.8500000000000001E-2</v>
@@ -1690,10 +1664,10 @@
         <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D43">
-        <v>0.15131889880952379</v>
+        <v>0.13817750946969701</v>
       </c>
       <c r="E43">
         <v>2.7E-2</v>
@@ -1719,10 +1693,10 @@
         <v>3</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D44">
-        <v>0.1573816785714286</v>
+        <v>0.14567057196969699</v>
       </c>
       <c r="E44">
         <v>3.6300000000000013E-2</v>
@@ -1748,10 +1722,10 @@
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D45">
-        <v>0.17578273809523809</v>
+        <v>0.16086837121212119</v>
       </c>
       <c r="E45">
         <v>3.5999999999999997E-2</v>
@@ -1780,22 +1754,22 @@
         <v>17</v>
       </c>
       <c r="D46">
-        <v>0.1854029166666667</v>
+        <v>0.17004025757575761</v>
       </c>
       <c r="E46">
-        <v>3.9E-2</v>
+        <v>3.7200000000000011E-2</v>
       </c>
       <c r="F46">
-        <v>9.1</v>
+        <v>6</v>
       </c>
       <c r="G46">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H46">
-        <v>13</v>
+        <v>12.4</v>
       </c>
       <c r="I46">
-        <v>3.71</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
@@ -1806,10 +1780,10 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D47">
-        <v>0.1372481190476191</v>
+        <v>0.1282402727272727</v>
       </c>
       <c r="E47">
         <v>3.0875E-2</v>
@@ -1835,10 +1809,10 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D48">
-        <v>0.16122514880952379</v>
+        <v>0.14711153724747481</v>
       </c>
       <c r="E48">
         <v>2.9250000000000009E-2</v>
@@ -1864,10 +1838,10 @@
         <v>3</v>
       </c>
       <c r="C49" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D49">
-        <v>0.16674867857142861</v>
+        <v>0.15423201641414139</v>
       </c>
       <c r="E49">
         <v>3.9325000000000013E-2</v>
@@ -1893,10 +1867,10 @@
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D50">
-        <v>0.1875327380952381</v>
+        <v>0.17150726010101011</v>
       </c>
       <c r="E50">
         <v>3.9000000000000007E-2</v>
@@ -1922,10 +1896,10 @@
         <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D51">
-        <v>0.19630541666666659</v>
+        <v>0.18118594065656571</v>
       </c>
       <c r="E51">
         <v>4.2250000000000003E-2</v>
@@ -1951,10 +1925,10 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D52">
-        <v>0.1435616190476191</v>
+        <v>0.1340537727272727</v>
       </c>
       <c r="E52">
         <v>3.3250000000000002E-2</v>
@@ -1980,10 +1954,10 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D53">
-        <v>0.1711313988095238</v>
+        <v>0.15604556502525249</v>
       </c>
       <c r="E53">
         <v>3.1500000000000007E-2</v>
@@ -2009,10 +1983,10 @@
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D54">
-        <v>0.17611567857142851</v>
+        <v>0.1627934608585859</v>
       </c>
       <c r="E54">
         <v>4.2350000000000013E-2</v>
@@ -2038,10 +2012,10 @@
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D55">
-        <v>0.19928273809523811</v>
+        <v>0.182146148989899</v>
       </c>
       <c r="E55">
         <v>4.2000000000000003E-2</v>
@@ -2070,22 +2044,22 @@
         <v>18</v>
       </c>
       <c r="D56">
-        <v>0.20415922619047619</v>
+        <v>0.19111621843434351</v>
       </c>
       <c r="E56">
-        <v>2.4500000000000001E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="F56">
-        <v>20</v>
+        <v>9.1</v>
       </c>
       <c r="G56">
-        <v>1.95</v>
+        <v>3.5</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I56">
-        <v>3.5897435897435899</v>
+        <v>3.71</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
@@ -2096,10 +2070,10 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D57">
-        <v>0.1498751190476191</v>
+        <v>0.1398672727272727</v>
       </c>
       <c r="E57">
         <v>3.5624999999999997E-2</v>
@@ -2125,10 +2099,10 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D58">
-        <v>0.1810376488095238</v>
+        <v>0.16497959280303029</v>
       </c>
       <c r="E58">
         <v>3.3750000000000002E-2</v>
@@ -2154,10 +2128,10 @@
         <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D59">
-        <v>0.18548267857142861</v>
+        <v>0.1713549053030303</v>
       </c>
       <c r="E59">
         <v>4.5375000000000013E-2</v>
@@ -2183,25 +2157,25 @@
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D60">
-        <v>0.21017485119047619</v>
+        <v>0.1927850378787879</v>
       </c>
       <c r="E60">
-        <v>2.6249999999999999E-2</v>
+        <v>4.5000000000000012E-2</v>
       </c>
       <c r="F60">
-        <v>20</v>
+        <v>5.8</v>
       </c>
       <c r="G60">
-        <v>1.95</v>
+        <v>4</v>
       </c>
       <c r="H60">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I60">
-        <v>3.5897435897435899</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
@@ -2215,7 +2189,7 @@
         <v>19</v>
       </c>
       <c r="D61">
-        <v>0.21017485119047619</v>
+        <v>0.19659801136363639</v>
       </c>
       <c r="E61">
         <v>2.6249999999999999E-2</v>
@@ -2241,10 +2215,10 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D62">
-        <v>0.1561886190476191</v>
+        <v>0.1456807727272727</v>
       </c>
       <c r="E62">
         <v>3.7999999999999999E-2</v>
@@ -2270,10 +2244,10 @@
         <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D63">
-        <v>0.19094389880952381</v>
+        <v>0.17391362058080809</v>
       </c>
       <c r="E63">
         <v>3.5999999999999997E-2</v>
@@ -2299,10 +2273,10 @@
         <v>3</v>
       </c>
       <c r="C64" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D64">
-        <v>0.19484967857142849</v>
+        <v>0.17991634974747481</v>
       </c>
       <c r="E64">
         <v>4.8400000000000012E-2</v>
@@ -2328,10 +2302,10 @@
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D65">
-        <v>0.21619047619047621</v>
+        <v>0.20207196969696969</v>
       </c>
       <c r="E65">
         <v>2.8000000000000001E-2</v>
@@ -2357,10 +2331,10 @@
         <v>5</v>
       </c>
       <c r="C66" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D66">
-        <v>0.21619047619047621</v>
+        <v>0.20207196969696969</v>
       </c>
       <c r="E66">
         <v>2.8000000000000001E-2</v>
@@ -2386,10 +2360,10 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D67">
-        <v>0.1625021190476191</v>
+        <v>0.1514942727272727</v>
       </c>
       <c r="E67">
         <v>4.0375000000000001E-2</v>
@@ -2415,10 +2389,10 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D68">
-        <v>0.20085014880952379</v>
+        <v>0.18284764835858591</v>
       </c>
       <c r="E68">
         <v>3.8250000000000013E-2</v>
@@ -2444,10 +2418,10 @@
         <v>3</v>
       </c>
       <c r="C69" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D69">
-        <v>0.2042166785714285</v>
+        <v>0.18847779419191921</v>
       </c>
       <c r="E69">
         <v>5.1425000000000012E-2</v>
@@ -2473,10 +2447,10 @@
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D70">
-        <v>0.22220610119047621</v>
+        <v>0.207545928030303</v>
       </c>
       <c r="E70">
         <v>2.9749999999999999E-2</v>
@@ -2502,10 +2476,10 @@
         <v>5</v>
       </c>
       <c r="C71" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D71">
-        <v>0.22220610119047621</v>
+        <v>0.207545928030303</v>
       </c>
       <c r="E71">
         <v>2.9749999999999999E-2</v>
@@ -2523,32 +2497,32 @@
         <v>3.5897435897435899</v>
       </c>
     </row>
-    <row r="72" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="2">
+    <row r="72" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
         <v>450</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="1">
         <v>1</v>
       </c>
-      <c r="C72" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72" s="2">
-        <v>0.1688156190476191</v>
-      </c>
-      <c r="E72" s="2">
+      <c r="C72" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="1">
+        <v>0.1573077727272727</v>
+      </c>
+      <c r="E72" s="1">
         <v>4.2750000000000003E-2</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>9.1999999999999993</v>
       </c>
-      <c r="G72" s="2">
+      <c r="G72" s="1">
         <v>1.8</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>9.5</v>
       </c>
-      <c r="I72" s="2">
+      <c r="I72" s="1">
         <v>5.28</v>
       </c>
     </row>
@@ -2560,10 +2534,10 @@
         <v>2</v>
       </c>
       <c r="C73" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D73">
-        <v>0.21075639880952379</v>
+        <v>0.19178167613636371</v>
       </c>
       <c r="E73">
         <v>4.0500000000000008E-2</v>
@@ -2589,10 +2563,10 @@
         <v>3</v>
       </c>
       <c r="C74" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D74">
-        <v>0.21358367857142849</v>
+        <v>0.19703923863636361</v>
       </c>
       <c r="E74">
         <v>5.4450000000000012E-2</v>
@@ -2618,10 +2592,10 @@
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D75">
-        <v>0.2282217261904762</v>
+        <v>0.21301988636363639</v>
       </c>
       <c r="E75">
         <v>3.15E-2</v>
@@ -2647,10 +2621,10 @@
         <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D76">
-        <v>0.2282217261904762</v>
+        <v>0.21301988636363639</v>
       </c>
       <c r="E76">
         <v>3.15E-2</v>
@@ -2676,10 +2650,10 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D77">
-        <v>0.1751291190476191</v>
+        <v>0.1631212727272727</v>
       </c>
       <c r="E77">
         <v>4.5124999999999998E-2</v>
@@ -2705,10 +2679,10 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D78">
-        <v>0.2206626488095238</v>
+        <v>0.2007157039141414</v>
       </c>
       <c r="E78">
         <v>4.2750000000000003E-2</v>
@@ -2734,10 +2708,10 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D79">
-        <v>0.2229506785714285</v>
+        <v>0.20560068308080809</v>
       </c>
       <c r="E79">
         <v>5.7475000000000012E-2</v>
@@ -2763,10 +2737,10 @@
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D80">
-        <v>0.2342373511904762</v>
+        <v>0.2184938446969697</v>
       </c>
       <c r="E80">
         <v>3.3250000000000002E-2</v>
@@ -2792,10 +2766,10 @@
         <v>5</v>
       </c>
       <c r="C81" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D81">
-        <v>0.2342373511904762</v>
+        <v>0.2184938446969697</v>
       </c>
       <c r="E81">
         <v>3.3250000000000002E-2</v>
@@ -2821,10 +2795,10 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D82">
-        <v>0.1814426190476191</v>
+        <v>0.1689347727272727</v>
       </c>
       <c r="E82">
         <v>4.7500000000000001E-2</v>
@@ -2850,10 +2824,10 @@
         <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D83">
-        <v>0.2305688988095238</v>
+        <v>0.20964973169191919</v>
       </c>
       <c r="E83">
         <v>4.5000000000000012E-2</v>
@@ -2879,10 +2853,10 @@
         <v>3</v>
       </c>
       <c r="C84" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D84">
-        <v>0.23231767857142849</v>
+        <v>0.21416212752525249</v>
       </c>
       <c r="E84">
         <v>6.0500000000000012E-2</v>
@@ -2908,10 +2882,10 @@
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D85">
-        <v>0.2402529761904762</v>
+        <v>0.22396780303030309</v>
       </c>
       <c r="E85">
         <v>3.5000000000000003E-2</v>
@@ -2937,10 +2911,10 @@
         <v>5</v>
       </c>
       <c r="C86" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D86">
-        <v>0.2402529761904762</v>
+        <v>0.22396780303030309</v>
       </c>
       <c r="E86">
         <v>3.5000000000000003E-2</v>
@@ -2966,10 +2940,10 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D87">
-        <v>0.1877561190476191</v>
+        <v>0.1747482727272727</v>
       </c>
       <c r="E87">
         <v>4.9875000000000003E-2</v>
@@ -2995,10 +2969,10 @@
         <v>2</v>
       </c>
       <c r="C88" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D88">
-        <v>0.24047514880952381</v>
+        <v>0.21858375946969699</v>
       </c>
       <c r="E88">
         <v>4.7250000000000007E-2</v>
@@ -3024,10 +2998,10 @@
         <v>3</v>
       </c>
       <c r="C89" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D89">
-        <v>0.24168467857142861</v>
+        <v>0.222723571969697</v>
       </c>
       <c r="E89">
         <v>6.3525000000000012E-2</v>
@@ -3053,10 +3027,10 @@
         <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D90">
-        <v>0.24626860119047619</v>
+        <v>0.22944176136363639</v>
       </c>
       <c r="E90">
         <v>3.6749999999999998E-2</v>
@@ -3082,10 +3056,10 @@
         <v>5</v>
       </c>
       <c r="C91" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D91">
-        <v>0.24626860119047619</v>
+        <v>0.22944176136363639</v>
       </c>
       <c r="E91">
         <v>3.6749999999999998E-2</v>
@@ -3111,10 +3085,10 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D92">
-        <v>0.1940696190476191</v>
+        <v>0.18056177272727281</v>
       </c>
       <c r="E92">
         <v>5.2249999999999998E-2</v>
@@ -3140,10 +3114,10 @@
         <v>2</v>
       </c>
       <c r="C93" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D93">
-        <v>0.25038139880952393</v>
+        <v>0.22751778724747479</v>
       </c>
       <c r="E93">
         <v>4.9500000000000009E-2</v>
@@ -3169,10 +3143,10 @@
         <v>3</v>
       </c>
       <c r="C94" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D94">
-        <v>0.25105167857142863</v>
+        <v>0.2312850164141414</v>
       </c>
       <c r="E94">
         <v>6.6550000000000012E-2</v>
@@ -3198,10 +3172,10 @@
         <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D95">
-        <v>0.25228422619047619</v>
+        <v>0.2349157196969697</v>
       </c>
       <c r="E95">
         <v>3.85E-2</v>
@@ -3227,10 +3201,10 @@
         <v>5</v>
       </c>
       <c r="C96" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D96">
-        <v>0.25228422619047619</v>
+        <v>0.2349157196969697</v>
       </c>
       <c r="E96">
         <v>3.85E-2</v>
@@ -3256,10 +3230,10 @@
         <v>1</v>
       </c>
       <c r="C97" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D97">
-        <v>0.2003831190476191</v>
+        <v>0.1863752727272727</v>
       </c>
       <c r="E97">
         <v>5.4625E-2</v>
@@ -3285,25 +3259,25 @@
         <v>2</v>
       </c>
       <c r="C98" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D98">
-        <v>0.25829985119047622</v>
+        <v>0.23645181502525259</v>
       </c>
       <c r="E98">
-        <v>4.0250000000000001E-2</v>
+        <v>5.1749999999999997E-2</v>
       </c>
       <c r="F98">
-        <v>20</v>
+        <v>5.41</v>
       </c>
       <c r="G98">
-        <v>1.95</v>
+        <v>3.5</v>
       </c>
       <c r="H98">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I98">
-        <v>3.5897435897435899</v>
+        <v>2.5714285714285721</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.35">
@@ -3314,25 +3288,25 @@
         <v>3</v>
       </c>
       <c r="C99" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D99">
-        <v>0.25829985119047622</v>
+        <v>0.23984646085858591</v>
       </c>
       <c r="E99">
-        <v>4.0250000000000001E-2</v>
+        <v>6.9575000000000012E-2</v>
       </c>
       <c r="F99">
-        <v>20</v>
+        <v>7.5</v>
       </c>
       <c r="G99">
-        <v>1.95</v>
+        <v>2.9</v>
       </c>
       <c r="H99">
-        <v>7</v>
+        <v>12.1</v>
       </c>
       <c r="I99">
-        <v>3.5897435897435899</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.35">
@@ -3343,25 +3317,25 @@
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D100">
-        <v>0.26028764880952387</v>
+        <v>0.24038967803030301</v>
       </c>
       <c r="E100">
-        <v>5.1749999999999997E-2</v>
+        <v>4.0250000000000001E-2</v>
       </c>
       <c r="F100">
-        <v>5.41</v>
+        <v>20</v>
       </c>
       <c r="G100">
-        <v>3.5</v>
+        <v>1.95</v>
       </c>
       <c r="H100">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I100">
-        <v>2.5714285714285721</v>
+        <v>3.5897435897435899</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.35">
@@ -3372,25 +3346,25 @@
         <v>5</v>
       </c>
       <c r="C101" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D101">
-        <v>0.26041867857142847</v>
+        <v>0.24038967803030301</v>
       </c>
       <c r="E101">
-        <v>6.9575000000000012E-2</v>
+        <v>4.0250000000000001E-2</v>
       </c>
       <c r="F101">
-        <v>7.5</v>
+        <v>20</v>
       </c>
       <c r="G101">
-        <v>2.9</v>
+        <v>1.95</v>
       </c>
       <c r="H101">
-        <v>12.1</v>
+        <v>7</v>
       </c>
       <c r="I101">
-        <v>4.17</v>
+        <v>3.5897435897435899</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.35">
@@ -3401,10 +3375,10 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D102">
-        <v>0.2066966190476191</v>
+        <v>0.19218877272727269</v>
       </c>
       <c r="E102">
         <v>5.7000000000000002E-2</v>
@@ -3430,25 +3404,25 @@
         <v>2</v>
       </c>
       <c r="C103" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D103">
-        <v>0.26431547619047618</v>
+        <v>0.2453858428030303</v>
       </c>
       <c r="E103">
-        <v>4.2000000000000003E-2</v>
+        <v>5.4000000000000013E-2</v>
       </c>
       <c r="F103">
-        <v>20</v>
+        <v>5.41</v>
       </c>
       <c r="G103">
-        <v>1.95</v>
+        <v>3.5</v>
       </c>
       <c r="H103">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I103">
-        <v>3.5897435897435899</v>
+        <v>2.5714285714285721</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.35">
@@ -3462,7 +3436,7 @@
         <v>19</v>
       </c>
       <c r="D104">
-        <v>0.26431547619047618</v>
+        <v>0.2458636363636364</v>
       </c>
       <c r="E104">
         <v>4.2000000000000003E-2</v>
@@ -3491,22 +3465,22 @@
         <v>20</v>
       </c>
       <c r="D105">
-        <v>0.26798452380952381</v>
+        <v>0.2458636363636364</v>
       </c>
       <c r="E105">
-        <v>4.6800000000000008E-2</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="F105">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G105">
-        <v>1.7</v>
+        <v>1.95</v>
       </c>
       <c r="H105">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="I105">
-        <v>4.5882352941176467</v>
+        <v>3.5897435897435899</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.35">
@@ -3517,25 +3491,25 @@
         <v>5</v>
       </c>
       <c r="C106" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D106">
-        <v>0.26800252380952377</v>
+        <v>0.24840790530303031</v>
       </c>
       <c r="E106">
-        <v>4.6800000000000008E-2</v>
+        <v>7.2600000000000012E-2</v>
       </c>
       <c r="F106">
-        <v>22</v>
+        <v>7.5</v>
       </c>
       <c r="G106">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="H106">
-        <v>7.8</v>
+        <v>12.1</v>
       </c>
       <c r="I106">
-        <v>4.59</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.35">
@@ -3546,10 +3520,10 @@
         <v>1</v>
       </c>
       <c r="C107" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D107">
-        <v>0.2130101190476191</v>
+        <v>0.19800227272727269</v>
       </c>
       <c r="E107">
         <v>5.9374999999999997E-2</v>
@@ -3575,10 +3549,10 @@
         <v>2</v>
       </c>
       <c r="C108" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D108">
-        <v>0.27033110119047621</v>
+        <v>0.2513375946969697</v>
       </c>
       <c r="E108">
         <v>4.3749999999999997E-2</v>
@@ -3604,10 +3578,10 @@
         <v>3</v>
       </c>
       <c r="C109" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D109">
-        <v>0.27033110119047621</v>
+        <v>0.2513375946969697</v>
       </c>
       <c r="E109">
         <v>4.3749999999999997E-2</v>
@@ -3633,25 +3607,25 @@
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D110">
-        <v>0.27365327380952381</v>
+        <v>0.25431987058080813</v>
       </c>
       <c r="E110">
-        <v>4.8750000000000009E-2</v>
+        <v>5.6250000000000008E-2</v>
       </c>
       <c r="F110">
-        <v>22</v>
+        <v>5.41</v>
       </c>
       <c r="G110">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="H110">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="I110">
-        <v>4.5882352941176467</v>
+        <v>2.5714285714285721</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.35">
@@ -3662,10 +3636,10 @@
         <v>5</v>
       </c>
       <c r="C111" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D111">
-        <v>0.27367202380952382</v>
+        <v>0.25585069444444453</v>
       </c>
       <c r="E111">
         <v>4.8750000000000009E-2</v>
@@ -3680,7 +3654,7 @@
         <v>7.8</v>
       </c>
       <c r="I111">
-        <v>4.59</v>
+        <v>4.5882352941176467</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.35">
@@ -3691,10 +3665,10 @@
         <v>1</v>
       </c>
       <c r="C112" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D112">
-        <v>0.2193236190476191</v>
+        <v>0.20381577272727269</v>
       </c>
       <c r="E112">
         <v>6.1749999999999999E-2</v>
@@ -3720,10 +3694,10 @@
         <v>2</v>
       </c>
       <c r="C113" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D113">
-        <v>0.27634672619047618</v>
+        <v>0.25681155303030301</v>
       </c>
       <c r="E113">
         <v>4.5500000000000013E-2</v>
@@ -3749,10 +3723,10 @@
         <v>3</v>
       </c>
       <c r="C114" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D114">
-        <v>0.27634672619047618</v>
+        <v>0.25681155303030301</v>
       </c>
       <c r="E114">
         <v>4.5500000000000013E-2</v>
@@ -3778,10 +3752,10 @@
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D115">
-        <v>0.27932202380952381</v>
+        <v>0.26104722222222221</v>
       </c>
       <c r="E115">
         <v>5.0700000000000009E-2</v>
@@ -3807,10 +3781,10 @@
         <v>5</v>
       </c>
       <c r="C116" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D116">
-        <v>0.27934152380952382</v>
+        <v>0.26106672222222232</v>
       </c>
       <c r="E116">
         <v>5.0700000000000009E-2</v>
@@ -3836,10 +3810,10 @@
         <v>1</v>
       </c>
       <c r="C117" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D117">
-        <v>0.2256371190476191</v>
+        <v>0.20962927272727269</v>
       </c>
       <c r="E117">
         <v>6.4125000000000001E-2</v>
@@ -3865,10 +3839,10 @@
         <v>2</v>
       </c>
       <c r="C118" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D118">
-        <v>0.2823623511904762</v>
+        <v>0.26228551136363643</v>
       </c>
       <c r="E118">
         <v>4.725E-2</v>
@@ -3894,10 +3868,10 @@
         <v>3</v>
       </c>
       <c r="C119" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D119">
-        <v>0.2823623511904762</v>
+        <v>0.26228551136363643</v>
       </c>
       <c r="E119">
         <v>4.725E-2</v>
@@ -3923,10 +3897,10 @@
         <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D120">
-        <v>0.28499077380952381</v>
+        <v>0.26624375</v>
       </c>
       <c r="E120">
         <v>5.2650000000000009E-2</v>
@@ -3952,10 +3926,10 @@
         <v>5</v>
       </c>
       <c r="C121" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D121">
-        <v>0.28501102380952381</v>
+        <v>0.26626400000000011</v>
       </c>
       <c r="E121">
         <v>5.2650000000000009E-2</v>
@@ -3981,10 +3955,10 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D122">
-        <v>0.2319506190476191</v>
+        <v>0.21544277272727269</v>
       </c>
       <c r="E122">
         <v>6.6500000000000004E-2</v>
@@ -4010,10 +3984,10 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D123">
-        <v>0.28837797619047623</v>
+        <v>0.26775946969696968</v>
       </c>
       <c r="E123">
         <v>4.9000000000000002E-2</v>
@@ -4039,10 +4013,10 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D124">
-        <v>0.28837797619047623</v>
+        <v>0.26775946969696968</v>
       </c>
       <c r="E124">
         <v>4.9000000000000002E-2</v>
@@ -4068,10 +4042,10 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D125">
-        <v>0.29065952380952381</v>
+        <v>0.27144027777777779</v>
       </c>
       <c r="E125">
         <v>5.460000000000001E-2</v>
@@ -4097,10 +4071,10 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D126">
-        <v>0.29068052380952381</v>
+        <v>0.27146127777777779</v>
       </c>
       <c r="E126">
         <v>5.460000000000001E-2</v>
@@ -4126,10 +4100,10 @@
         <v>1</v>
       </c>
       <c r="C127" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D127">
-        <v>0.2382641190476191</v>
+        <v>0.22125627272727269</v>
       </c>
       <c r="E127">
         <v>6.8875000000000006E-2</v>
@@ -4155,10 +4129,10 @@
         <v>2</v>
       </c>
       <c r="C128" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D128">
-        <v>0.2943936011904762</v>
+        <v>0.27323342803030298</v>
       </c>
       <c r="E128">
         <v>5.0750000000000003E-2</v>
@@ -4184,10 +4158,10 @@
         <v>3</v>
       </c>
       <c r="C129" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D129">
-        <v>0.2943936011904762</v>
+        <v>0.27323342803030298</v>
       </c>
       <c r="E129">
         <v>5.0750000000000003E-2</v>
@@ -4213,10 +4187,10 @@
         <v>4</v>
       </c>
       <c r="C130" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D130">
-        <v>0.29632827380952381</v>
+        <v>0.27663680555555559</v>
       </c>
       <c r="E130">
         <v>5.655000000000001E-2</v>
@@ -4242,10 +4216,10 @@
         <v>5</v>
       </c>
       <c r="C131" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D131">
-        <v>0.2963500238095238</v>
+        <v>0.27665855555555557</v>
       </c>
       <c r="E131">
         <v>5.655000000000001E-2</v>
@@ -4271,10 +4245,10 @@
         <v>1</v>
       </c>
       <c r="C132" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D132">
-        <v>0.2445776190476191</v>
+        <v>0.22706977272727269</v>
       </c>
       <c r="E132">
         <v>7.1250000000000008E-2</v>
@@ -4300,10 +4274,10 @@
         <v>2</v>
       </c>
       <c r="C133" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D133">
-        <v>0.30040922619047622</v>
+        <v>0.27870738636363629</v>
       </c>
       <c r="E133">
         <v>5.2499999999999998E-2</v>
@@ -4329,10 +4303,10 @@
         <v>3</v>
       </c>
       <c r="C134" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D134">
-        <v>0.30040922619047622</v>
+        <v>0.27870738636363629</v>
       </c>
       <c r="E134">
         <v>5.2499999999999998E-2</v>
@@ -4358,10 +4332,10 @@
         <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D135">
-        <v>0.30199702380952381</v>
+        <v>0.28183333333333338</v>
       </c>
       <c r="E135">
         <v>5.850000000000001E-2</v>
@@ -4387,10 +4361,10 @@
         <v>5</v>
       </c>
       <c r="C136" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D136">
-        <v>0.30201952380952379</v>
+        <v>0.28185583333333342</v>
       </c>
       <c r="E136">
         <v>5.850000000000001E-2</v>
@@ -4416,10 +4390,10 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D137">
-        <v>0.25089111904761913</v>
+        <v>0.23288327272727269</v>
       </c>
       <c r="E137">
         <v>7.3624999999999996E-2</v>
@@ -4445,10 +4419,10 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D138">
-        <v>0.30642485119047619</v>
+        <v>0.28418134469696971</v>
       </c>
       <c r="E138">
         <v>5.4250000000000007E-2</v>
@@ -4474,10 +4448,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D139">
-        <v>0.30642485119047619</v>
+        <v>0.28418134469696971</v>
       </c>
       <c r="E139">
         <v>5.4250000000000007E-2</v>
@@ -4503,10 +4477,10 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D140">
-        <v>0.30766577380952381</v>
+        <v>0.28702986111111112</v>
       </c>
       <c r="E140">
         <v>6.0450000000000011E-2</v>
@@ -4532,10 +4506,10 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D141">
-        <v>0.30768902380952379</v>
+        <v>0.28705311111111109</v>
       </c>
       <c r="E141">
         <v>6.0450000000000011E-2</v>
@@ -4561,10 +4535,10 @@
         <v>1</v>
       </c>
       <c r="C142" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D142">
-        <v>0.2572046190476191</v>
+        <v>0.23869677272727269</v>
       </c>
       <c r="E142">
         <v>7.5999999999999998E-2</v>
@@ -4590,10 +4564,10 @@
         <v>2</v>
       </c>
       <c r="C143" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D143">
-        <v>0.31244047619047621</v>
+        <v>0.28965530303030312</v>
       </c>
       <c r="E143">
         <v>5.6000000000000001E-2</v>
@@ -4619,10 +4593,10 @@
         <v>3</v>
       </c>
       <c r="C144" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D144">
-        <v>0.31244047619047621</v>
+        <v>0.28965530303030312</v>
       </c>
       <c r="E144">
         <v>5.6000000000000001E-2</v>
@@ -4648,10 +4622,10 @@
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D145">
-        <v>0.31333452380952381</v>
+        <v>0.29222638888888891</v>
       </c>
       <c r="E145">
         <v>6.2400000000000011E-2</v>
@@ -4677,10 +4651,10 @@
         <v>5</v>
       </c>
       <c r="C146" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D146">
-        <v>0.31335852380952378</v>
+        <v>0.29225038888888888</v>
       </c>
       <c r="E146">
         <v>6.2400000000000011E-2</v>

</xml_diff>